<commit_message>
eval: 完整评测报告更新 — Intent 98.8% / SubScenario 70.5% / ALL PASS
全场景评测 (86条合成用例):
- Intent 准确率: 98.8% (PASS ≥80%)
- SubScenario 准确率: 70.5% (PASS ≥70%)
- 回复安全: 100%
- P95 延迟: 4.8s (PASS <10s)

食安分类评测 (200条真实用例):
- 精确率: 100% (零误报)
- 召回率: 64% (FN主要为上下文缺失的"转人工"类消息)
- 子场景准确率: 82.8%

🤖 Generated with [Qoder][https://qoder.com]
</commit_message>
<xml_diff>
--- a/classification_eval_v5.xlsx
+++ b/classification_eval_v5.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1647" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="260">
   <si>
     <t>index</t>
   </si>
@@ -597,6 +597,9 @@
     <t>general_food_safety</t>
   </si>
   <si>
+    <t>browse_menu</t>
+  </si>
+  <si>
     <t>delivery_issue</t>
   </si>
   <si>
@@ -604,9 +607,6 @@
   </si>
   <si>
     <t>taste_issue</t>
-  </si>
-  <si>
-    <t>browse_menu</t>
   </si>
   <si>
     <t>spoilage</t>
@@ -2320,7 +2320,10 @@
         <v>185</v>
       </c>
       <c r="D40" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E40" t="s">
+        <v>193</v>
       </c>
       <c r="F40" t="s">
         <v>199</v>
@@ -2549,7 +2552,7 @@
         <v>185</v>
       </c>
       <c r="E48" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F48" t="s">
         <v>199</v>
@@ -2828,7 +2831,7 @@
         <v>185</v>
       </c>
       <c r="E57" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F57" t="s">
         <v>199</v>
@@ -2915,7 +2918,10 @@
         <v>185</v>
       </c>
       <c r="D60" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E60" t="s">
+        <v>193</v>
       </c>
       <c r="F60" t="s">
         <v>199</v>
@@ -2941,7 +2947,7 @@
         <v>185</v>
       </c>
       <c r="D61" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E61" t="s">
         <v>193</v>
@@ -3275,7 +3281,7 @@
         <v>185</v>
       </c>
       <c r="E72" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F72" t="s">
         <v>201</v>
@@ -3388,7 +3394,7 @@
         <v>186</v>
       </c>
       <c r="E76" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F76" t="s">
         <v>200</v>
@@ -3661,7 +3667,7 @@
         <v>187</v>
       </c>
       <c r="E85" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F85" t="s">
         <v>200</v>
@@ -3806,7 +3812,7 @@
         <v>186</v>
       </c>
       <c r="E90" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F90" t="s">
         <v>200</v>
@@ -4189,7 +4195,10 @@
         <v>185</v>
       </c>
       <c r="D103" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E103" t="s">
+        <v>193</v>
       </c>
       <c r="F103" t="s">
         <v>199</v>
@@ -4509,7 +4518,7 @@
         <v>187</v>
       </c>
       <c r="E113" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F113" t="s">
         <v>199</v>
@@ -5034,10 +5043,10 @@
         <v>185</v>
       </c>
       <c r="D131" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E131" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F131" t="s">
         <v>199</v>
@@ -5231,7 +5240,10 @@
         <v>185</v>
       </c>
       <c r="D138" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E138" t="s">
+        <v>193</v>
       </c>
       <c r="F138" t="s">
         <v>199</v>
@@ -5971,7 +5983,10 @@
         <v>186</v>
       </c>
       <c r="D163" t="s">
-        <v>185</v>
+        <v>186</v>
+      </c>
+      <c r="E163" t="s">
+        <v>192</v>
       </c>
       <c r="F163" t="s">
         <v>200</v>
@@ -5986,7 +6001,10 @@
         <v>230</v>
       </c>
       <c r="J163" t="s">
-        <v>249</v>
+        <v>250</v>
+      </c>
+      <c r="K163" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="164" spans="1:11">
@@ -6296,7 +6314,10 @@
         <v>185</v>
       </c>
       <c r="D174" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E174" t="s">
+        <v>193</v>
       </c>
       <c r="F174" t="s">
         <v>199</v>
@@ -7003,7 +7024,10 @@
         <v>185</v>
       </c>
       <c r="D199" t="s">
-        <v>185</v>
+        <v>187</v>
+      </c>
+      <c r="E199" t="s">
+        <v>193</v>
       </c>
       <c r="F199" t="s">
         <v>199</v>

</xml_diff>